<commit_message>
Implement equipment cards and rewire catalog workbook
</commit_message>
<xml_diff>
--- a/catalogue_astronomie.xlsx
+++ b/catalogue_astronomie.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Derfence\Documents\Gatcha\client-android-standalone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0618CF5-FAFB-42B7-84BC-EDF44201BAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D430C3D1-E14E-42C9-A4BC-18A8404374E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogue" sheetId="1" r:id="rId1"/>
-    <sheet name="Donnees" sheetId="2" r:id="rId2"/>
-    <sheet name="Resultats" sheetId="3" r:id="rId3"/>
+    <sheet name="Equipements" sheetId="4" r:id="rId2"/>
+    <sheet name="Donnees" sheetId="2" r:id="rId3"/>
+    <sheet name="Resultats" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1617" uniqueCount="795">
   <si>
     <t>rowType</t>
   </si>
@@ -2286,6 +2287,162 @@
   </si>
   <si>
     <t>percentEpicPerDay</t>
+  </si>
+  <si>
+    <t>equipmentCardId</t>
+  </si>
+  <si>
+    <t>equipmentType</t>
+  </si>
+  <si>
+    <t>displayName</t>
+  </si>
+  <si>
+    <t>level</t>
+  </si>
+  <si>
+    <t>packsAffected</t>
+  </si>
+  <si>
+    <t>bonusValue</t>
+  </si>
+  <si>
+    <t>bonusUnit</t>
+  </si>
+  <si>
+    <t>dropWeight</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>observatory-beginner</t>
+  </si>
+  <si>
+    <t>observatory</t>
+  </si>
+  <si>
+    <t>Observatoire debutant</t>
+  </si>
+  <si>
+    <t>equipment_observatory_1</t>
+  </si>
+  <si>
+    <t>rechargeMultiplier</t>
+  </si>
+  <si>
+    <t>Accelere legerement la recharge des packs.</t>
+  </si>
+  <si>
+    <t>observatory-advanced</t>
+  </si>
+  <si>
+    <t>Observatoire expert</t>
+  </si>
+  <si>
+    <t>equipment_observatory_2</t>
+  </si>
+  <si>
+    <t>Maintient une recharge plus rapide pendant plusieurs packs.</t>
+  </si>
+  <si>
+    <t>observatory-master</t>
+  </si>
+  <si>
+    <t>Observatoire legendaire</t>
+  </si>
+  <si>
+    <t>equipment_observatory_3</t>
+  </si>
+  <si>
+    <t>Double la vitesse de recharge pour une courte serie de packs.</t>
+  </si>
+  <si>
+    <t>telescope-beginner</t>
+  </si>
+  <si>
+    <t>telescope</t>
+  </si>
+  <si>
+    <t>Telescope debutant</t>
+  </si>
+  <si>
+    <t>equipment_telescope_1</t>
+  </si>
+  <si>
+    <t>holographicPercent</t>
+  </si>
+  <si>
+    <t>Ajoute une petite chance holographique supplementaire.</t>
+  </si>
+  <si>
+    <t>telescope-advanced</t>
+  </si>
+  <si>
+    <t>Telescope expert</t>
+  </si>
+  <si>
+    <t>equipment_telescope_2</t>
+  </si>
+  <si>
+    <t>Renforce sensiblement l'apparition des cartes holographiques.</t>
+  </si>
+  <si>
+    <t>telescope-master</t>
+  </si>
+  <si>
+    <t>Telescope legendaire</t>
+  </si>
+  <si>
+    <t>equipment_telescope_3</t>
+  </si>
+  <si>
+    <t>Offre une forte poussee holographique sur les prochains packs.</t>
+  </si>
+  <si>
+    <t>mount-beginner</t>
+  </si>
+  <si>
+    <t>mount</t>
+  </si>
+  <si>
+    <t>Monture debutante</t>
+  </si>
+  <si>
+    <t>equipment_mount_1</t>
+  </si>
+  <si>
+    <t>rarityBoost</t>
+  </si>
+  <si>
+    <t>Ajoute une chance moderee de promouvoir une carte d'un palier.</t>
+  </si>
+  <si>
+    <t>mount-advanced</t>
+  </si>
+  <si>
+    <t>Monture experte</t>
+  </si>
+  <si>
+    <t>equipment_mount_2</t>
+  </si>
+  <si>
+    <t>Augmente davantage la probabilite de gagner en rarete.</t>
+  </si>
+  <si>
+    <t>mount-master</t>
+  </si>
+  <si>
+    <t>Monture legendaire</t>
+  </si>
+  <si>
+    <t>equipment_mount_3</t>
+  </si>
+  <si>
+    <t>Pousse les tirages vers des cartes plus rares pendant plusieurs packs.</t>
+  </si>
+  <si>
+    <t>EquipmentChancePercent</t>
   </si>
 </sst>
 </file>
@@ -9488,8 +9645,350 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4D42EB6-033C-42BF-9E1D-DED894C3BFBF}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="64.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1" t="s">
+        <v>744</v>
+      </c>
+      <c r="C1" t="s">
+        <v>745</v>
+      </c>
+      <c r="D1" t="s">
+        <v>746</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>747</v>
+      </c>
+      <c r="G1" t="s">
+        <v>748</v>
+      </c>
+      <c r="H1" t="s">
+        <v>749</v>
+      </c>
+      <c r="I1" t="s">
+        <v>750</v>
+      </c>
+      <c r="J1" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>752</v>
+      </c>
+      <c r="B2" t="s">
+        <v>753</v>
+      </c>
+      <c r="C2" t="s">
+        <v>754</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>755</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>1.25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>756</v>
+      </c>
+      <c r="I2">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>758</v>
+      </c>
+      <c r="B3" t="s">
+        <v>753</v>
+      </c>
+      <c r="C3" t="s">
+        <v>759</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>760</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>1.5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>756</v>
+      </c>
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="J3" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>762</v>
+      </c>
+      <c r="B4" t="s">
+        <v>753</v>
+      </c>
+      <c r="C4" t="s">
+        <v>763</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>764</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4" t="s">
+        <v>756</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
+      <c r="J4" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>766</v>
+      </c>
+      <c r="B5" t="s">
+        <v>767</v>
+      </c>
+      <c r="C5" t="s">
+        <v>768</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>769</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>8</v>
+      </c>
+      <c r="H5" t="s">
+        <v>770</v>
+      </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>772</v>
+      </c>
+      <c r="B6" t="s">
+        <v>767</v>
+      </c>
+      <c r="C6" t="s">
+        <v>773</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>774</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
+        <v>770</v>
+      </c>
+      <c r="I6">
+        <v>10</v>
+      </c>
+      <c r="J6" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>776</v>
+      </c>
+      <c r="B7" t="s">
+        <v>767</v>
+      </c>
+      <c r="C7" t="s">
+        <v>777</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>778</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>18</v>
+      </c>
+      <c r="H7" t="s">
+        <v>770</v>
+      </c>
+      <c r="I7">
+        <v>4</v>
+      </c>
+      <c r="J7" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>780</v>
+      </c>
+      <c r="B8" t="s">
+        <v>781</v>
+      </c>
+      <c r="C8" t="s">
+        <v>782</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>783</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8">
+        <v>6</v>
+      </c>
+      <c r="H8" t="s">
+        <v>784</v>
+      </c>
+      <c r="I8">
+        <v>16</v>
+      </c>
+      <c r="J8" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>786</v>
+      </c>
+      <c r="B9" t="s">
+        <v>781</v>
+      </c>
+      <c r="C9" t="s">
+        <v>787</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>788</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="G9">
+        <v>10</v>
+      </c>
+      <c r="H9" t="s">
+        <v>784</v>
+      </c>
+      <c r="I9">
+        <v>10</v>
+      </c>
+      <c r="J9" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>790</v>
+      </c>
+      <c r="B10" t="s">
+        <v>781</v>
+      </c>
+      <c r="C10" t="s">
+        <v>791</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>792</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>784</v>
+      </c>
+      <c r="I10">
+        <v>4</v>
+      </c>
+      <c r="J10" t="s">
+        <v>793</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -9677,12 +10176,20 @@
         <v>10</v>
       </c>
     </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>794</v>
+      </c>
+      <c r="B19" s="2">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Sync catalog workbook updates
</commit_message>
<xml_diff>
--- a/catalogue_astronomie.xlsx
+++ b/catalogue_astronomie.xlsx
@@ -9119,7 +9119,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dobson</t>
+          <t xml:space="preserve">Newton</t>
         </is>
       </c>
       <c r="D5">
@@ -11914,7 +11914,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dobson</t>
+          <t xml:space="preserve">Newton</t>
         </is>
       </c>
       <c r="D79">

</xml_diff>

<commit_message>
Ameliore les indicateurs du menu equipement
</commit_message>
<xml_diff>
--- a/catalogue_astronomie.xlsx
+++ b/catalogue_astronomie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Derfence\Documents\Gatcha\client-android-standalone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8143B11E-62EE-46C9-AAA3-7D6E492D7768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0C60F9-ADB5-499E-B840-E99AB75AE156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalogue" sheetId="1" r:id="rId1"/>
@@ -2223,9 +2223,6 @@
     <t>equipment_mount_3</t>
   </si>
   <si>
-    <t>Pousse les tirages vers des cartes plus rares pendant plusieurs packs.</t>
-  </si>
-  <si>
     <t>EquipmentChancePercent</t>
   </si>
   <si>
@@ -2470,6 +2467,9 @@
   </si>
   <si>
     <t>holographicSkyPercent</t>
+  </si>
+  <si>
+    <t>Améliore grandement la probabilité de gagner en rareté.</t>
   </si>
 </sst>
 </file>
@@ -3668,7 +3668,7 @@
         <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G3" t="s">
         <v>52</v>
@@ -3683,7 +3683,7 @@
         <v>54</v>
       </c>
       <c r="K3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="L3" t="s">
         <v>55</v>
@@ -3734,7 +3734,7 @@
         <v>64</v>
       </c>
       <c r="AB3" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="AC3" t="s">
         <v>57</v>
@@ -3835,7 +3835,7 @@
         <v>78</v>
       </c>
       <c r="AB4" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="AC4" t="s">
         <v>57</v>
@@ -3936,7 +3936,7 @@
         <v>89</v>
       </c>
       <c r="AB5" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="AC5" t="s">
         <v>57</v>
@@ -3971,7 +3971,7 @@
         <v>93</v>
       </c>
       <c r="F6" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G6" t="s">
         <v>52</v>
@@ -3986,7 +3986,7 @@
         <v>54</v>
       </c>
       <c r="K6" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="L6" t="s">
         <v>55</v>
@@ -4037,7 +4037,7 @@
         <v>100</v>
       </c>
       <c r="AB6" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="AC6" t="s">
         <v>57</v>
@@ -4072,7 +4072,7 @@
         <v>104</v>
       </c>
       <c r="F7" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="G7" t="s">
         <v>52</v>
@@ -4087,7 +4087,7 @@
         <v>54</v>
       </c>
       <c r="K7" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="L7" t="s">
         <v>106</v>
@@ -4138,7 +4138,7 @@
         <v>111</v>
       </c>
       <c r="AB7" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="AC7" t="s">
         <v>15</v>
@@ -4254,7 +4254,7 @@
         <v>124</v>
       </c>
       <c r="AB8" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="AC8" t="s">
         <v>57</v>
@@ -4289,7 +4289,7 @@
         <v>127</v>
       </c>
       <c r="F9" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="G9" t="s">
         <v>128</v>
@@ -4304,7 +4304,7 @@
         <v>54</v>
       </c>
       <c r="K9" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="L9" t="s">
         <v>130</v>
@@ -4405,7 +4405,7 @@
         <v>142</v>
       </c>
       <c r="F10" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="G10" t="s">
         <v>52</v>
@@ -4420,7 +4420,7 @@
         <v>54</v>
       </c>
       <c r="K10" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="L10" t="s">
         <v>55</v>
@@ -4471,7 +4471,7 @@
         <v>150</v>
       </c>
       <c r="AB10" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="AC10" t="s">
         <v>57</v>
@@ -4572,7 +4572,7 @@
         <v>162</v>
       </c>
       <c r="AB11" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="AC11" t="s">
         <v>57</v>
@@ -4607,7 +4607,7 @@
         <v>166</v>
       </c>
       <c r="F12" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="G12" t="s">
         <v>52</v>
@@ -4622,7 +4622,7 @@
         <v>54</v>
       </c>
       <c r="K12" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="L12" t="s">
         <v>106</v>
@@ -4673,7 +4673,7 @@
         <v>171</v>
       </c>
       <c r="AB12" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="AC12" t="s">
         <v>15</v>
@@ -4857,7 +4857,7 @@
         <v>191</v>
       </c>
       <c r="F14" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="G14" t="s">
         <v>128</v>
@@ -4872,7 +4872,7 @@
         <v>54</v>
       </c>
       <c r="K14" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="L14" t="s">
         <v>193</v>
@@ -5056,7 +5056,7 @@
         <v>208</v>
       </c>
       <c r="F16" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="G16" t="s">
         <v>52</v>
@@ -5071,7 +5071,7 @@
         <v>54</v>
       </c>
       <c r="K16" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="L16" t="s">
         <v>210</v>
@@ -5122,7 +5122,7 @@
         <v>215</v>
       </c>
       <c r="AB16" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="AC16" t="s">
         <v>180</v>
@@ -5190,7 +5190,7 @@
         <v>222</v>
       </c>
       <c r="F17" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="G17" t="s">
         <v>52</v>
@@ -5205,7 +5205,7 @@
         <v>54</v>
       </c>
       <c r="K17" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="L17" t="s">
         <v>106</v>
@@ -5306,7 +5306,7 @@
         <v>231</v>
       </c>
       <c r="F18" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="G18" t="s">
         <v>70</v>
@@ -5321,7 +5321,7 @@
         <v>54</v>
       </c>
       <c r="K18" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="L18" t="s">
         <v>233</v>
@@ -5422,7 +5422,7 @@
         <v>241</v>
       </c>
       <c r="F19" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G19" t="s">
         <v>128</v>
@@ -5437,7 +5437,7 @@
         <v>54</v>
       </c>
       <c r="K19" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="L19" t="s">
         <v>243</v>
@@ -5571,7 +5571,7 @@
         <v>255</v>
       </c>
       <c r="AB20" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="AC20" t="s">
         <v>180</v>
@@ -5639,7 +5639,7 @@
         <v>259</v>
       </c>
       <c r="F21" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="G21" t="s">
         <v>70</v>
@@ -5654,7 +5654,7 @@
         <v>54</v>
       </c>
       <c r="K21" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="L21" t="s">
         <v>233</v>
@@ -5705,7 +5705,7 @@
         <v>264</v>
       </c>
       <c r="AB21" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="AC21" t="s">
         <v>132</v>
@@ -5937,7 +5937,7 @@
         <v>284</v>
       </c>
       <c r="AB23" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="AC23" t="s">
         <v>180</v>
@@ -6139,7 +6139,7 @@
         <v>304</v>
       </c>
       <c r="F25" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="G25" t="s">
         <v>305</v>
@@ -6154,7 +6154,7 @@
         <v>54</v>
       </c>
       <c r="K25" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="L25" t="s">
         <v>278</v>
@@ -6205,7 +6205,7 @@
         <v>312</v>
       </c>
       <c r="AB25" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="AC25" t="s">
         <v>180</v>
@@ -6273,7 +6273,7 @@
         <v>318</v>
       </c>
       <c r="F26" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="G26" t="s">
         <v>305</v>
@@ -6288,7 +6288,7 @@
         <v>54</v>
       </c>
       <c r="K26" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="L26" t="s">
         <v>278</v>
@@ -6339,7 +6339,7 @@
         <v>325</v>
       </c>
       <c r="AB26" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="AC26" t="s">
         <v>180</v>
@@ -6473,7 +6473,7 @@
         <v>336</v>
       </c>
       <c r="AB27" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="AC27" t="s">
         <v>180</v>
@@ -6556,7 +6556,7 @@
         <v>54</v>
       </c>
       <c r="K28" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="L28" t="s">
         <v>278</v>
@@ -6607,7 +6607,7 @@
         <v>348</v>
       </c>
       <c r="AB28" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="AC28" t="s">
         <v>180</v>
@@ -6669,7 +6669,7 @@
         <v>353</v>
       </c>
       <c r="F29" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G29" t="s">
         <v>70</v>
@@ -6684,7 +6684,7 @@
         <v>54</v>
       </c>
       <c r="K29" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="L29" t="s">
         <v>278</v>
@@ -6803,7 +6803,7 @@
         <v>366</v>
       </c>
       <c r="F30" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G30" t="s">
         <v>52</v>
@@ -6818,7 +6818,7 @@
         <v>54</v>
       </c>
       <c r="K30" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="L30" t="s">
         <v>278</v>
@@ -6869,7 +6869,7 @@
         <v>372</v>
       </c>
       <c r="AB30" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="AC30" t="s">
         <v>180</v>
@@ -7003,7 +7003,7 @@
         <v>384</v>
       </c>
       <c r="AB31" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="AC31" t="s">
         <v>180</v>
@@ -7137,7 +7137,7 @@
         <v>396</v>
       </c>
       <c r="AB32" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="AC32" t="s">
         <v>180</v>
@@ -7271,7 +7271,7 @@
         <v>405</v>
       </c>
       <c r="AB33" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="AC33" t="s">
         <v>180</v>
@@ -7405,7 +7405,7 @@
         <v>415</v>
       </c>
       <c r="AB34" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="AC34" t="s">
         <v>180</v>
@@ -7607,7 +7607,7 @@
         <v>430</v>
       </c>
       <c r="F36" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G36" t="s">
         <v>52</v>
@@ -7622,7 +7622,7 @@
         <v>54</v>
       </c>
       <c r="K36" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="L36" t="s">
         <v>278</v>
@@ -7673,7 +7673,7 @@
         <v>436</v>
       </c>
       <c r="AB36" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="AC36" t="s">
         <v>180</v>
@@ -7741,7 +7741,7 @@
         <v>442</v>
       </c>
       <c r="F37" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="G37" t="s">
         <v>52</v>
@@ -7756,7 +7756,7 @@
         <v>54</v>
       </c>
       <c r="K37" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="L37" t="s">
         <v>278</v>
@@ -7807,7 +7807,7 @@
         <v>447</v>
       </c>
       <c r="AB37" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="AC37" t="s">
         <v>180</v>
@@ -7941,7 +7941,7 @@
         <v>459</v>
       </c>
       <c r="AB38" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="AC38" t="s">
         <v>180</v>
@@ -8009,7 +8009,7 @@
         <v>464</v>
       </c>
       <c r="F39" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="G39" t="s">
         <v>305</v>
@@ -8024,7 +8024,7 @@
         <v>54</v>
       </c>
       <c r="K39" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="L39" t="s">
         <v>278</v>
@@ -8209,7 +8209,7 @@
         <v>482</v>
       </c>
       <c r="AB40" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="AC40" t="s">
         <v>180</v>
@@ -8292,7 +8292,7 @@
         <v>54</v>
       </c>
       <c r="K41" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="L41" t="s">
         <v>278</v>
@@ -8846,7 +8846,7 @@
         <v>546</v>
       </c>
       <c r="AB45" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="AC45" t="s">
         <v>57</v>
@@ -8881,7 +8881,7 @@
         <v>549</v>
       </c>
       <c r="F46" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="G46" t="s">
         <v>305</v>
@@ -8896,7 +8896,7 @@
         <v>54</v>
       </c>
       <c r="K46" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="L46" t="s">
         <v>551</v>
@@ -8947,7 +8947,7 @@
         <v>555</v>
       </c>
       <c r="AB46" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="AC46" t="s">
         <v>180</v>
@@ -9131,7 +9131,7 @@
         <v>568</v>
       </c>
       <c r="F48" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="G48" t="s">
         <v>52</v>
@@ -9146,7 +9146,7 @@
         <v>54</v>
       </c>
       <c r="K48" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="L48" t="s">
         <v>233</v>
@@ -9197,7 +9197,7 @@
         <v>573</v>
       </c>
       <c r="AB48" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="AC48" t="s">
         <v>132</v>
@@ -9247,7 +9247,7 @@
         <v>574</v>
       </c>
       <c r="F49" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="G49" t="s">
         <v>52</v>
@@ -9262,7 +9262,7 @@
         <v>54</v>
       </c>
       <c r="K49" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="L49" t="s">
         <v>106</v>
@@ -9363,7 +9363,7 @@
         <v>580</v>
       </c>
       <c r="F50" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="G50" t="s">
         <v>52</v>
@@ -9378,7 +9378,7 @@
         <v>54</v>
       </c>
       <c r="K50" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="L50" t="s">
         <v>55</v>
@@ -9429,7 +9429,7 @@
         <v>588</v>
       </c>
       <c r="AB50" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="AC50" t="s">
         <v>57</v>
@@ -9735,7 +9735,7 @@
         <v>697</v>
       </c>
       <c r="C2" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -9756,7 +9756,7 @@
         <v>16</v>
       </c>
       <c r="J2" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -9767,7 +9767,7 @@
         <v>697</v>
       </c>
       <c r="C3" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -9799,7 +9799,7 @@
         <v>697</v>
       </c>
       <c r="C4" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="D4">
         <v>3</v>
@@ -9820,7 +9820,7 @@
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -9831,7 +9831,7 @@
         <v>706</v>
       </c>
       <c r="C5" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -9846,13 +9846,13 @@
         <v>8</v>
       </c>
       <c r="H5" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="I5">
         <v>16</v>
       </c>
       <c r="J5" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -9863,7 +9863,7 @@
         <v>706</v>
       </c>
       <c r="C6" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -9878,7 +9878,7 @@
         <v>12</v>
       </c>
       <c r="H6" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="I6">
         <v>10</v>
@@ -9895,7 +9895,7 @@
         <v>706</v>
       </c>
       <c r="C7" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="D7">
         <v>3</v>
@@ -9910,13 +9910,13 @@
         <v>18</v>
       </c>
       <c r="H7" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="I7">
         <v>4</v>
       </c>
       <c r="J7" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -9927,7 +9927,7 @@
         <v>714</v>
       </c>
       <c r="C8" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -9948,7 +9948,7 @@
         <v>16</v>
       </c>
       <c r="J8" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -9959,7 +9959,7 @@
         <v>714</v>
       </c>
       <c r="C9" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -9980,7 +9980,7 @@
         <v>10</v>
       </c>
       <c r="J9" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -9991,7 +9991,7 @@
         <v>714</v>
       </c>
       <c r="C10" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="D10">
         <v>3</v>
@@ -10012,7 +10012,7 @@
         <v>4</v>
       </c>
       <c r="J10" t="s">
-        <v>721</v>
+        <v>803</v>
       </c>
     </row>
   </sheetData>
@@ -10097,19 +10097,19 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="B10" s="2">
         <f>1/7</f>
         <v>0.14285714285714285</v>
       </c>
       <c r="D10" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B11" s="1">
         <f>D4-B12</f>
@@ -10121,7 +10121,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B12" s="1">
         <f>D11*D4/100</f>
@@ -10219,7 +10219,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
@@ -10656,31 +10656,31 @@
         <v>658</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="K19" s="9" t="s">
         <v>659</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="M19" s="11" t="s">
         <v>660</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="O19" s="5" t="s">
         <v>661</v>
       </c>
       <c r="P19" s="5" t="s">
+        <v>799</v>
+      </c>
+      <c r="Q19" s="16" t="s">
         <v>800</v>
       </c>
-      <c r="Q19" s="16" t="s">
+      <c r="R19" s="16" t="s">
         <v>801</v>
-      </c>
-      <c r="R19" s="16" t="s">
-        <v>802</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
@@ -10691,7 +10691,7 @@
         <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D20" t="s">
         <v>52</v>
@@ -10901,7 +10901,7 @@
         <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="D23" t="s">
         <v>52</v>
@@ -10971,7 +10971,7 @@
         <v>104</v>
       </c>
       <c r="C24" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D24" t="s">
         <v>52</v>
@@ -11111,7 +11111,7 @@
         <v>127</v>
       </c>
       <c r="C26" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="D26" t="s">
         <v>128</v>
@@ -11181,7 +11181,7 @@
         <v>142</v>
       </c>
       <c r="C27" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D27" t="s">
         <v>52</v>
@@ -11321,7 +11321,7 @@
         <v>166</v>
       </c>
       <c r="C29" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D29" t="s">
         <v>52</v>
@@ -11461,7 +11461,7 @@
         <v>191</v>
       </c>
       <c r="C31" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D31" t="s">
         <v>128</v>
@@ -11601,7 +11601,7 @@
         <v>208</v>
       </c>
       <c r="C33" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D33" t="s">
         <v>52</v>
@@ -11671,7 +11671,7 @@
         <v>222</v>
       </c>
       <c r="C34" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="D34" t="s">
         <v>52</v>
@@ -11741,7 +11741,7 @@
         <v>231</v>
       </c>
       <c r="C35" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="D35" t="s">
         <v>70</v>
@@ -11811,7 +11811,7 @@
         <v>241</v>
       </c>
       <c r="C36" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="D36" t="s">
         <v>128</v>
@@ -11951,7 +11951,7 @@
         <v>259</v>
       </c>
       <c r="C38" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="D38" t="s">
         <v>70</v>
@@ -12231,7 +12231,7 @@
         <v>304</v>
       </c>
       <c r="C42" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="D42" t="s">
         <v>305</v>
@@ -12301,7 +12301,7 @@
         <v>318</v>
       </c>
       <c r="C43" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="D43" t="s">
         <v>305</v>
@@ -12511,7 +12511,7 @@
         <v>353</v>
       </c>
       <c r="C46" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D46" t="s">
         <v>70</v>
@@ -12581,7 +12581,7 @@
         <v>366</v>
       </c>
       <c r="C47" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="D47" t="s">
         <v>52</v>
@@ -13001,7 +13001,7 @@
         <v>430</v>
       </c>
       <c r="C53" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D53" t="s">
         <v>52</v>
@@ -13071,7 +13071,7 @@
         <v>442</v>
       </c>
       <c r="C54" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="D54" t="s">
         <v>52</v>
@@ -13211,7 +13211,7 @@
         <v>464</v>
       </c>
       <c r="C56" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="D56" t="s">
         <v>305</v>
@@ -13701,7 +13701,7 @@
         <v>549</v>
       </c>
       <c r="C63" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D63" t="s">
         <v>305</v>
@@ -13841,7 +13841,7 @@
         <v>568</v>
       </c>
       <c r="C65" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D65" t="s">
         <v>52</v>
@@ -13911,7 +13911,7 @@
         <v>574</v>
       </c>
       <c r="C66" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="D66" t="s">
         <v>52</v>
@@ -13981,7 +13981,7 @@
         <v>580</v>
       </c>
       <c r="C67" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="D67" t="s">
         <v>52</v>

</xml_diff>